<commit_message>
ran the site level statistical tests for the carbon stock and carbon content
</commit_message>
<xml_diff>
--- a/data/carbon/Aveiro2025_Biomass_C_cores.xlsx
+++ b/data/carbon/Aveiro2025_Biomass_C_cores.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\REWRITE\Field_data\Nantes_cloud\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\REWRITE\Field_data\seagrass_carbon_2025\data\carbon\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="4" r:id="rId1"/>
@@ -17,6 +17,7 @@
     <sheet name="seagrass biomass" sheetId="2" r:id="rId3"/>
     <sheet name="carbon" sheetId="5" r:id="rId4"/>
     <sheet name="moisture" sheetId="6" r:id="rId5"/>
+    <sheet name="soil" sheetId="7" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">raw!$A$1:$O$100</definedName>
@@ -25,7 +26,7 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -160,7 +161,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2136" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2159" uniqueCount="591">
   <si>
     <t>type</t>
   </si>
@@ -2021,6 +2022,72 @@
   </si>
   <si>
     <t>RR_39_B</t>
+  </si>
+  <si>
+    <t>Petri_dish</t>
+  </si>
+  <si>
+    <t>Init_weight_petri</t>
+  </si>
+  <si>
+    <t>Final_weight_petri</t>
+  </si>
+  <si>
+    <t>RS01</t>
+  </si>
+  <si>
+    <t>RS02</t>
+  </si>
+  <si>
+    <t>RS03</t>
+  </si>
+  <si>
+    <t>RS04</t>
+  </si>
+  <si>
+    <t>RS05</t>
+  </si>
+  <si>
+    <t>RS06</t>
+  </si>
+  <si>
+    <t>RS07</t>
+  </si>
+  <si>
+    <t>RS08</t>
+  </si>
+  <si>
+    <t>NS01</t>
+  </si>
+  <si>
+    <t>NS02</t>
+  </si>
+  <si>
+    <t>NS03</t>
+  </si>
+  <si>
+    <t>NS04</t>
+  </si>
+  <si>
+    <t>NS05</t>
+  </si>
+  <si>
+    <t>NS06</t>
+  </si>
+  <si>
+    <t>NS07</t>
+  </si>
+  <si>
+    <t>NS08</t>
+  </si>
+  <si>
+    <t>Init_weight</t>
+  </si>
+  <si>
+    <t>Final_weight</t>
+  </si>
+  <si>
+    <t>Dry_bulk_density</t>
   </si>
 </sst>
 </file>
@@ -2758,6 +2825,27 @@
     <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="10" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="1" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2771,27 +2859,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="4" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="10" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -22675,78 +22742,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="87"/>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
-      <c r="D1" s="88" t="s">
+      <c r="A1" s="78"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="79" t="s">
         <v>457</v>
       </c>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="79"/>
       <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="87"/>
-      <c r="B2" s="87"/>
-      <c r="C2" s="87"/>
-      <c r="D2" s="88" t="s">
+      <c r="A2" s="78"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="79" t="s">
         <v>458</v>
       </c>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88"/>
-      <c r="H2" s="88"/>
-      <c r="I2" s="88"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
       <c r="J2" s="32"/>
     </row>
     <row r="3" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="87"/>
-      <c r="B3" s="87"/>
-      <c r="C3" s="87"/>
-      <c r="D3" s="89" t="s">
+      <c r="A3" s="78"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="80" t="s">
         <v>459</v>
       </c>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
       <c r="J3" s="32"/>
     </row>
     <row r="5" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="83" t="s">
+      <c r="A5" s="81" t="s">
         <v>460</v>
       </c>
-      <c r="B5" s="83"/>
-      <c r="C5" s="85"/>
-      <c r="D5" s="85"/>
+      <c r="B5" s="81"/>
+      <c r="C5" s="82"/>
+      <c r="D5" s="82"/>
     </row>
     <row r="6" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="83" t="s">
+      <c r="A6" s="81" t="s">
         <v>461</v>
       </c>
-      <c r="B6" s="83"/>
-      <c r="C6" s="84"/>
-      <c r="D6" s="84"/>
+      <c r="B6" s="81"/>
+      <c r="C6" s="83"/>
+      <c r="D6" s="83"/>
     </row>
     <row r="7" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="83" t="s">
+      <c r="A7" s="81" t="s">
         <v>462</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="85"/>
-      <c r="D7" s="85"/>
+      <c r="B7" s="81"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
     </row>
     <row r="8" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="83" t="s">
+      <c r="A8" s="81" t="s">
         <v>463</v>
       </c>
-      <c r="B8" s="83"/>
-      <c r="C8" s="86"/>
-      <c r="D8" s="86"/>
+      <c r="B8" s="81"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="84"/>
     </row>
     <row r="9" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="34"/>
@@ -22759,62 +22826,62 @@
     </row>
     <row r="10" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="35"/>
-      <c r="B10" s="79" t="s">
+      <c r="B10" s="86" t="s">
         <v>464</v>
       </c>
-      <c r="C10" s="79"/>
-      <c r="D10" s="79"/>
-      <c r="E10" s="79"/>
-      <c r="F10" s="79" t="s">
+      <c r="C10" s="86"/>
+      <c r="D10" s="86"/>
+      <c r="E10" s="86"/>
+      <c r="F10" s="86" t="s">
         <v>465</v>
       </c>
-      <c r="G10" s="79"/>
-      <c r="H10" s="79"/>
-      <c r="I10" s="79"/>
+      <c r="G10" s="86"/>
+      <c r="H10" s="86"/>
+      <c r="I10" s="86"/>
     </row>
     <row r="11" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="80" t="s">
+      <c r="A11" s="87" t="s">
         <v>466</v>
       </c>
-      <c r="B11" s="81" t="s">
+      <c r="B11" s="88" t="s">
         <v>467</v>
       </c>
-      <c r="C11" s="78" t="s">
+      <c r="C11" s="85" t="s">
         <v>468</v>
       </c>
-      <c r="D11" s="82" t="s">
+      <c r="D11" s="89" t="s">
         <v>469</v>
       </c>
-      <c r="E11" s="78" t="s">
+      <c r="E11" s="85" t="s">
         <v>470</v>
       </c>
-      <c r="F11" s="82" t="s">
+      <c r="F11" s="89" t="s">
         <v>467</v>
       </c>
-      <c r="G11" s="78" t="s">
+      <c r="G11" s="85" t="s">
         <v>468</v>
       </c>
-      <c r="H11" s="78" t="s">
+      <c r="H11" s="85" t="s">
         <v>471</v>
       </c>
-      <c r="I11" s="78" t="s">
+      <c r="I11" s="85" t="s">
         <v>472</v>
       </c>
-      <c r="J11" s="78" t="s">
+      <c r="J11" s="85" t="s">
         <v>473</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="80"/>
-      <c r="B12" s="81"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="82"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="82"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
+      <c r="A12" s="87"/>
+      <c r="B12" s="88"/>
+      <c r="C12" s="85"/>
+      <c r="D12" s="89"/>
+      <c r="E12" s="85"/>
+      <c r="F12" s="89"/>
+      <c r="G12" s="85"/>
+      <c r="H12" s="85"/>
+      <c r="I12" s="85"/>
+      <c r="J12" s="85"/>
     </row>
     <row r="13" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="36"/>
@@ -24707,11 +24774,11 @@
         <v>1.8839999999999999</v>
       </c>
       <c r="I72" s="51">
-        <f t="shared" ref="I72:I76" si="22">(H72*1000/F72)*G72</f>
+        <f>(H72*1000/F72)*G72</f>
         <v>8.3285442730206434</v>
       </c>
       <c r="J72" s="48">
-        <f t="shared" ref="J72:J76" si="23">E72-I72</f>
+        <f>E72-I72</f>
         <v>310.70210433710048</v>
       </c>
     </row>
@@ -24742,11 +24809,11 @@
         <v>1.0369999999999999</v>
       </c>
       <c r="I73" s="51">
-        <f t="shared" si="22"/>
+        <f>(H73*1000/F73)*G73</f>
         <v>5.1700069797586998</v>
       </c>
       <c r="J73" s="48">
-        <f t="shared" si="23"/>
+        <f>E73-I73</f>
         <v>289.61156253292222</v>
       </c>
     </row>
@@ -24777,11 +24844,11 @@
         <v>0.2777</v>
       </c>
       <c r="I74" s="51">
-        <f t="shared" si="22"/>
+        <f>(H74*1000/F74)*G74</f>
         <v>1.3652900688298917</v>
       </c>
       <c r="J74" s="48">
-        <f t="shared" si="23"/>
+        <f>E74-I74</f>
         <v>321.24652660703981</v>
       </c>
     </row>
@@ -24812,11 +24879,11 @@
         <v>0.6583</v>
       </c>
       <c r="I75" s="51">
-        <f t="shared" si="22"/>
+        <f>(H75*1000/F75)*G75</f>
         <v>3.1652081930954901</v>
       </c>
       <c r="J75" s="48">
-        <f t="shared" si="23"/>
+        <f>E75-I75</f>
         <v>295.78539329141944</v>
       </c>
     </row>
@@ -24847,11 +24914,11 @@
         <v>0.94920000000000004</v>
       </c>
       <c r="I76" s="51">
-        <f t="shared" si="22"/>
+        <f>(H76*1000/F76)*G76</f>
         <v>4.3298969072164954</v>
       </c>
       <c r="J76" s="48">
-        <f t="shared" si="23"/>
+        <f>E76-I76</f>
         <v>283.95711386986801</v>
       </c>
     </row>
@@ -24894,11 +24961,11 @@
         <v>0.74280000000000002</v>
       </c>
       <c r="I78" s="51">
-        <f t="shared" ref="I78:I82" si="24">(H78*1000/F78)*G78</f>
+        <f>(H78*1000/F78)*G78</f>
         <v>3.166510358939381</v>
       </c>
       <c r="J78" s="48">
-        <f t="shared" ref="J78:J82" si="25">E78-I78</f>
+        <f>E78-I78</f>
         <v>235.58683895709504</v>
       </c>
     </row>
@@ -24929,11 +24996,11 @@
         <v>0.46689999999999998</v>
       </c>
       <c r="I79" s="51">
-        <f t="shared" si="24"/>
+        <f>(H79*1000/F79)*G79</f>
         <v>2.3009067612852356</v>
       </c>
       <c r="J79" s="48">
-        <f t="shared" si="25"/>
+        <f>E79-I79</f>
         <v>263.1545562717705</v>
       </c>
     </row>
@@ -24964,11 +25031,11 @@
         <v>0.93279999999999996</v>
       </c>
       <c r="I80" s="51">
-        <f t="shared" si="24"/>
+        <f>(H80*1000/F80)*G80</f>
         <v>4.2911031373631427</v>
       </c>
       <c r="J80" s="48">
-        <f t="shared" si="25"/>
+        <f>E80-I80</f>
         <v>219.27763902728373</v>
       </c>
     </row>
@@ -24999,11 +25066,11 @@
         <v>0.83840000000000003</v>
       </c>
       <c r="I81" s="51">
-        <f t="shared" si="24"/>
+        <f>(H81*1000/F81)*G81</f>
         <v>3.9053474939444759</v>
       </c>
       <c r="J81" s="48">
-        <f t="shared" si="25"/>
+        <f>E81-I81</f>
         <v>248.96673202070636</v>
       </c>
     </row>
@@ -25034,11 +25101,11 @@
         <v>1.0329999999999999</v>
       </c>
       <c r="I82" s="51">
-        <f t="shared" si="24"/>
+        <f>(H82*1000/F82)*G82</f>
         <v>4.6460376000719616</v>
       </c>
       <c r="J82" s="48">
-        <f t="shared" si="25"/>
+        <f>E82-I82</f>
         <v>251.28818862987103</v>
       </c>
     </row>
@@ -25081,11 +25148,11 @@
         <v>1.6120000000000001</v>
       </c>
       <c r="I84" s="51">
-        <f t="shared" ref="I84:I92" si="26">(H84*1000/F84)*G84</f>
+        <f t="shared" ref="I84:I92" si="22">(H84*1000/F84)*G84</f>
         <v>7.9679699471108698</v>
       </c>
       <c r="J84" s="48">
-        <f t="shared" ref="J84:J92" si="27">E84-I84</f>
+        <f t="shared" ref="J84:J92" si="23">E84-I84</f>
         <v>276.25763901472317</v>
       </c>
     </row>
@@ -25116,11 +25183,11 @@
         <v>0.40550000000000003</v>
       </c>
       <c r="I85" s="51">
-        <f t="shared" si="26"/>
+        <f t="shared" si="22"/>
         <v>1.9974385498251319</v>
       </c>
       <c r="J85" s="48">
-        <f t="shared" si="27"/>
+        <f t="shared" si="23"/>
         <v>277.33532933256112</v>
       </c>
     </row>
@@ -25151,11 +25218,11 @@
         <v>1.333</v>
       </c>
       <c r="I86" s="51">
-        <f t="shared" si="26"/>
+        <f t="shared" si="22"/>
         <v>6.3494331713822998</v>
       </c>
       <c r="J86" s="48">
-        <f t="shared" si="27"/>
+        <f t="shared" si="23"/>
         <v>296.51888495117311</v>
       </c>
     </row>
@@ -25186,11 +25253,11 @@
         <v>0</v>
       </c>
       <c r="I87" s="51">
-        <f t="shared" si="26"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="J87" s="48">
-        <f t="shared" si="27"/>
+        <f t="shared" si="23"/>
         <v>285.69436698271056</v>
       </c>
     </row>
@@ -25233,11 +25300,11 @@
         <v>1.1459999999999999</v>
       </c>
       <c r="I89" s="51">
-        <f t="shared" si="26"/>
+        <f t="shared" si="22"/>
         <v>5.6741100163390605</v>
       </c>
       <c r="J89" s="48">
-        <f t="shared" si="27"/>
+        <f t="shared" si="23"/>
         <v>225.10577639452117</v>
       </c>
     </row>
@@ -25268,11 +25335,11 @@
         <v>0.25940000000000002</v>
       </c>
       <c r="I90" s="51">
-        <f t="shared" si="26"/>
+        <f t="shared" si="22"/>
         <v>1.2227774111435847</v>
       </c>
       <c r="J90" s="48">
-        <f t="shared" si="27"/>
+        <f t="shared" si="23"/>
         <v>238.24916978357587</v>
       </c>
     </row>
@@ -25303,11 +25370,11 @@
         <v>0.2412</v>
       </c>
       <c r="I91" s="51">
-        <f t="shared" si="26"/>
+        <f t="shared" si="22"/>
         <v>1.1922886801779533</v>
       </c>
       <c r="J91" s="48">
-        <f t="shared" si="27"/>
+        <f t="shared" si="23"/>
         <v>238.08280688827739</v>
       </c>
     </row>
@@ -25338,11 +25405,11 @@
         <v>0</v>
       </c>
       <c r="I92" s="51">
-        <f t="shared" si="26"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="J92" s="48">
-        <f t="shared" si="27"/>
+        <f t="shared" si="23"/>
         <v>194.70649895178198</v>
       </c>
     </row>
@@ -25365,18 +25432,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:C3"/>
-    <mergeCell ref="D1:I1"/>
-    <mergeCell ref="D2:I2"/>
-    <mergeCell ref="D3:I3"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
     <mergeCell ref="I11:I12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="B10:E10"/>
@@ -25389,6 +25444,18 @@
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="G11:G12"/>
     <mergeCell ref="H11:H12"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="A1:C3"/>
+    <mergeCell ref="D1:I1"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.23611111111111099" right="0.23611111111111099" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="81" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -25792,4 +25859,461 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>557</v>
+      </c>
+      <c r="B1" t="s">
+        <v>569</v>
+      </c>
+      <c r="C1" t="s">
+        <v>570</v>
+      </c>
+      <c r="D1" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1" t="s">
+        <v>588</v>
+      </c>
+      <c r="F1" t="s">
+        <v>589</v>
+      </c>
+      <c r="G1" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>572</v>
+      </c>
+      <c r="B2">
+        <v>8.4529999999999994</v>
+      </c>
+      <c r="C2">
+        <v>39.57</v>
+      </c>
+      <c r="D2">
+        <v>27.128</v>
+      </c>
+      <c r="E2">
+        <f>C2-$B2</f>
+        <v>31.117000000000001</v>
+      </c>
+      <c r="F2">
+        <f>D2-$B2</f>
+        <v>18.675000000000001</v>
+      </c>
+      <c r="G2">
+        <f>F2/20</f>
+        <v>0.93375000000000008</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>573</v>
+      </c>
+      <c r="B3">
+        <v>7.3449999999999998</v>
+      </c>
+      <c r="C3">
+        <v>36.25</v>
+      </c>
+      <c r="D3">
+        <v>25.039000000000001</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E17" si="0">C3-$B3</f>
+        <v>28.905000000000001</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F17" si="1">D3-$B3</f>
+        <v>17.694000000000003</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G17" si="2">F3/20</f>
+        <v>0.88470000000000015</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>574</v>
+      </c>
+      <c r="B4">
+        <v>8.3119999999999994</v>
+      </c>
+      <c r="C4">
+        <v>40.463000000000001</v>
+      </c>
+      <c r="D4">
+        <v>29.382999999999999</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>32.151000000000003</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="1"/>
+        <v>21.070999999999998</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="2"/>
+        <v>1.05355</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>575</v>
+      </c>
+      <c r="B5">
+        <v>7.1029999999999998</v>
+      </c>
+      <c r="C5">
+        <v>35.981999999999999</v>
+      </c>
+      <c r="D5">
+        <v>24.556999999999999</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>28.878999999999998</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>17.454000000000001</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="2"/>
+        <v>0.87270000000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>576</v>
+      </c>
+      <c r="B6">
+        <v>8.4369999999999994</v>
+      </c>
+      <c r="C6">
+        <v>68.662999999999997</v>
+      </c>
+      <c r="D6">
+        <v>26.135999999999999</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>60.225999999999999</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>17.698999999999998</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="2"/>
+        <v>0.8849499999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>577</v>
+      </c>
+      <c r="B7">
+        <v>7.3289999999999997</v>
+      </c>
+      <c r="C7">
+        <v>32.713000000000001</v>
+      </c>
+      <c r="D7">
+        <v>21.346</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>25.384</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>14.016999999999999</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="2"/>
+        <v>0.70084999999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>578</v>
+      </c>
+      <c r="B8">
+        <v>8.32</v>
+      </c>
+      <c r="C8">
+        <v>37.764000000000003</v>
+      </c>
+      <c r="D8">
+        <v>25.591999999999999</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>29.444000000000003</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>17.271999999999998</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="2"/>
+        <v>0.86359999999999992</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>579</v>
+      </c>
+      <c r="B9">
+        <v>8.4390000000000001</v>
+      </c>
+      <c r="C9">
+        <v>34.822000000000003</v>
+      </c>
+      <c r="D9">
+        <v>25.2</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>26.383000000000003</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="1"/>
+        <v>16.760999999999999</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="2"/>
+        <v>0.83804999999999996</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>580</v>
+      </c>
+      <c r="B10">
+        <v>7.1150000000000002</v>
+      </c>
+      <c r="C10">
+        <v>36.137</v>
+      </c>
+      <c r="D10">
+        <v>23.271999999999998</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>29.021999999999998</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>16.156999999999996</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="2"/>
+        <v>0.80784999999999985</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>581</v>
+      </c>
+      <c r="B11">
+        <v>8.3239999999999998</v>
+      </c>
+      <c r="C11">
+        <v>37.029000000000003</v>
+      </c>
+      <c r="D11">
+        <v>24.58</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>28.705000000000005</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>16.256</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="2"/>
+        <v>0.81279999999999997</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>582</v>
+      </c>
+      <c r="B12">
+        <v>7.3310000000000004</v>
+      </c>
+      <c r="C12">
+        <v>37.670999999999999</v>
+      </c>
+      <c r="D12">
+        <v>25.385000000000002</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>30.34</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>18.054000000000002</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="2"/>
+        <v>0.90270000000000006</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>583</v>
+      </c>
+      <c r="B13">
+        <v>7.1120000000000001</v>
+      </c>
+      <c r="C13">
+        <v>36.411999999999999</v>
+      </c>
+      <c r="D13">
+        <v>23.952000000000002</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>29.299999999999997</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>16.840000000000003</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="2"/>
+        <v>0.84200000000000019</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>584</v>
+      </c>
+      <c r="B14">
+        <v>7.1059999999999999</v>
+      </c>
+      <c r="C14">
+        <v>36.823999999999998</v>
+      </c>
+      <c r="D14">
+        <v>24.004000000000001</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>29.717999999999996</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>16.898000000000003</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="2"/>
+        <v>0.84490000000000021</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>585</v>
+      </c>
+      <c r="B15">
+        <v>8.3140000000000001</v>
+      </c>
+      <c r="C15">
+        <v>36.771000000000001</v>
+      </c>
+      <c r="D15">
+        <v>24.411000000000001</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>28.457000000000001</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>16.097000000000001</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="2"/>
+        <v>0.80485000000000007</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>586</v>
+      </c>
+      <c r="B16">
+        <v>7.3310000000000004</v>
+      </c>
+      <c r="C16">
+        <v>36.93</v>
+      </c>
+      <c r="D16">
+        <v>24.879000000000001</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>29.599</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="1"/>
+        <v>17.548000000000002</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="2"/>
+        <v>0.87740000000000007</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>587</v>
+      </c>
+      <c r="B17">
+        <v>8.44</v>
+      </c>
+      <c r="C17">
+        <v>38.298999999999999</v>
+      </c>
+      <c r="D17">
+        <v>26.274000000000001</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>29.859000000000002</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="1"/>
+        <v>17.834000000000003</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="2"/>
+        <v>0.89170000000000016</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>